<commit_message>
chore: checkpoint — strip real-file metadata from the Excel fixture
Caught while preparing the first push: the sanitized workbook still carried
lastModifiedBy with a real name and a sheet named after the real query. Names
and CPFs had been replaced, but document properties had not, and publishing to
a public remote would have carried them out of the machine.

The generator now renames the sheet and runs Excel's own Document Inspector
removal before saving, so the file stays Excel-written and no longer says who
produced it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/pgfn/lista-manual.xlsx
+++ b/fixtures/pgfn/lista-manual.xlsx
@@ -2,18 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damaz\AppData\Local\Temp\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{49C5052E-3A5B-4059-8BCA-2C9E97F88C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B17F5C39-A7EE-4B0F-B391-CAD435ADA061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB8E60DC-E9D1-463A-90F5-714B4C83A492}"/>
   </bookViews>
   <sheets>
-    <sheet name="Consulta_Lista_Devedores_2026_0" sheetId="1" r:id="rId1"/>
+    <sheet name="Lista" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>